<commit_message>
comentarios da funcao 2 e aumento da funcao 3 em txt pra excel
</commit_message>
<xml_diff>
--- a/testes/silicone_smf_5pontos/media_dos_5pontos.xlsx
+++ b/testes/silicone_smf_5pontos/media_dos_5pontos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -554,1270 +554,1317 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2.114</v>
+        <v>1.139</v>
       </c>
       <c r="B3" t="n">
-        <v>2.4025</v>
+        <v>0.5589999999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>3.43</v>
+        <v>0.869</v>
       </c>
       <c r="D3" t="n">
-        <v>3.431999999999999</v>
+        <v>0.985</v>
       </c>
       <c r="E3" t="n">
-        <v>4.318</v>
+        <v>1.356</v>
       </c>
       <c r="F3" t="n">
-        <v>5.390000000000001</v>
+        <v>1.328</v>
       </c>
       <c r="G3" t="n">
-        <v>6.51</v>
+        <v>2.554</v>
       </c>
       <c r="H3" t="n">
-        <v>6.51</v>
+        <v>2.175</v>
       </c>
       <c r="I3" t="n">
-        <v>7.802</v>
+        <v>2.777</v>
       </c>
       <c r="J3" t="n">
-        <v>8.006</v>
+        <v>2.845</v>
       </c>
       <c r="K3" t="n">
-        <v>8.146000000000001</v>
+        <v>2.877</v>
       </c>
       <c r="L3" t="n">
-        <v>8.98</v>
+        <v>4.29</v>
       </c>
       <c r="M3" t="n">
-        <v>9.596</v>
+        <v>4.851000000000001</v>
       </c>
       <c r="N3" t="n">
-        <v>10.396</v>
+        <v>5.151999999999999</v>
       </c>
       <c r="O3" t="n">
-        <v>12.19</v>
+        <v>6.268000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1.93</v>
+        <v>2.114</v>
       </c>
       <c r="B4" t="n">
-        <v>2.706</v>
+        <v>2.4025</v>
       </c>
       <c r="C4" t="n">
-        <v>3.18</v>
+        <v>3.43</v>
       </c>
       <c r="D4" t="n">
-        <v>3.582</v>
+        <v>3.431999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>4.198</v>
+        <v>4.318</v>
       </c>
       <c r="F4" t="n">
-        <v>4.668</v>
+        <v>5.390000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>5.497999999999999</v>
+        <v>6.51</v>
       </c>
       <c r="H4" t="n">
-        <v>5.642</v>
+        <v>6.51</v>
       </c>
       <c r="I4" t="n">
-        <v>6.178</v>
+        <v>7.802</v>
       </c>
       <c r="J4" t="n">
-        <v>6.286</v>
+        <v>8.006</v>
       </c>
       <c r="K4" t="n">
-        <v>7.025999999999999</v>
+        <v>8.146000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>7.544</v>
+        <v>8.98</v>
       </c>
       <c r="M4" t="n">
-        <v>7.718000000000001</v>
+        <v>9.596</v>
       </c>
       <c r="N4" t="n">
-        <v>8.24</v>
+        <v>10.396</v>
       </c>
       <c r="O4" t="n">
-        <v>8.914</v>
+        <v>12.19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2.114</v>
+        <v>1.93</v>
       </c>
       <c r="B5" t="n">
-        <v>2.607</v>
+        <v>2.706</v>
       </c>
       <c r="C5" t="n">
-        <v>3.43</v>
+        <v>3.18</v>
       </c>
       <c r="D5" t="n">
-        <v>3.431999999999999</v>
+        <v>3.582</v>
       </c>
       <c r="E5" t="n">
-        <v>4.318</v>
+        <v>4.198</v>
       </c>
       <c r="F5" t="n">
-        <v>5.390000000000001</v>
+        <v>4.668</v>
       </c>
       <c r="G5" t="n">
-        <v>6.51</v>
+        <v>5.497999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>6.51</v>
+        <v>5.642</v>
       </c>
       <c r="I5" t="n">
-        <v>7.802</v>
+        <v>6.178</v>
       </c>
       <c r="J5" t="n">
-        <v>8.006</v>
+        <v>6.286</v>
       </c>
       <c r="K5" t="n">
-        <v>8.146000000000001</v>
+        <v>7.025999999999999</v>
       </c>
       <c r="L5" t="n">
-        <v>8.98</v>
+        <v>7.544</v>
       </c>
       <c r="M5" t="n">
-        <v>9.596</v>
+        <v>7.718000000000001</v>
       </c>
       <c r="N5" t="n">
-        <v>10.396</v>
+        <v>8.24</v>
       </c>
       <c r="O5" t="n">
-        <v>12.19</v>
+        <v>8.914</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2.259</v>
+        <v>2.114</v>
       </c>
       <c r="B6" t="n">
-        <v>2.7405</v>
+        <v>2.607</v>
       </c>
       <c r="C6" t="n">
-        <v>3.966</v>
+        <v>3.43</v>
       </c>
       <c r="D6" t="n">
-        <v>4.166</v>
+        <v>3.431999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>5.138</v>
+        <v>4.318</v>
       </c>
       <c r="F6" t="n">
-        <v>6.318</v>
+        <v>5.390000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>7.465999999999999</v>
+        <v>6.51</v>
       </c>
       <c r="H6" t="n">
-        <v>7.512</v>
+        <v>6.51</v>
       </c>
       <c r="I6" t="n">
-        <v>8.84</v>
+        <v>7.802</v>
       </c>
       <c r="J6" t="n">
-        <v>9.449999999999999</v>
+        <v>8.006</v>
       </c>
       <c r="K6" t="n">
-        <v>9.528</v>
+        <v>8.146000000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>10.52</v>
+        <v>8.98</v>
       </c>
       <c r="M6" t="n">
-        <v>11.014</v>
+        <v>9.596</v>
       </c>
       <c r="N6" t="n">
-        <v>12.076</v>
+        <v>10.396</v>
       </c>
       <c r="O6" t="n">
-        <v>14.01</v>
+        <v>12.19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2.004</v>
+        <v>2.259</v>
       </c>
       <c r="B7" t="n">
-        <v>2.684</v>
+        <v>2.7405</v>
       </c>
       <c r="C7" t="n">
-        <v>4.076</v>
+        <v>3.966</v>
       </c>
       <c r="D7" t="n">
-        <v>4.48</v>
+        <v>4.166</v>
       </c>
       <c r="E7" t="n">
-        <v>5.27</v>
+        <v>5.138</v>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>6.318</v>
       </c>
       <c r="G7" t="n">
-        <v>8.017999999999999</v>
+        <v>7.465999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>8.406000000000001</v>
+        <v>7.512</v>
       </c>
       <c r="I7" t="n">
-        <v>9.826000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="J7" t="n">
-        <v>10.468</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>10.734</v>
+        <v>9.528</v>
       </c>
       <c r="L7" t="n">
-        <v>11.704</v>
+        <v>10.52</v>
       </c>
       <c r="M7" t="n">
-        <v>12.5</v>
+        <v>11.014</v>
       </c>
       <c r="N7" t="n">
-        <v>13.482</v>
+        <v>12.076</v>
       </c>
       <c r="O7" t="n">
-        <v>15.498</v>
+        <v>14.01</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2.22</v>
+        <v>2.004</v>
       </c>
       <c r="B8" t="n">
-        <v>3.048</v>
+        <v>2.684</v>
       </c>
       <c r="C8" t="n">
-        <v>4.03</v>
+        <v>4.076</v>
       </c>
       <c r="D8" t="n">
-        <v>5.322</v>
+        <v>4.48</v>
       </c>
       <c r="E8" t="n">
-        <v>6.228</v>
+        <v>5.27</v>
       </c>
       <c r="F8" t="n">
-        <v>7.692</v>
+        <v>7</v>
       </c>
       <c r="G8" t="n">
-        <v>9.093999999999999</v>
+        <v>8.017999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>9.284000000000001</v>
+        <v>8.406000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>10.854</v>
+        <v>9.826000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>11.584</v>
+        <v>10.468</v>
       </c>
       <c r="K8" t="n">
-        <v>12.022</v>
+        <v>10.734</v>
       </c>
       <c r="L8" t="n">
-        <v>13.19</v>
+        <v>11.704</v>
       </c>
       <c r="M8" t="n">
-        <v>13.948</v>
+        <v>12.5</v>
       </c>
       <c r="N8" t="n">
-        <v>14.874</v>
+        <v>13.482</v>
       </c>
       <c r="O8" t="n">
-        <v>17.054</v>
+        <v>15.498</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2.714</v>
+        <v>2.22</v>
       </c>
       <c r="B9" t="n">
-        <v>3.654</v>
+        <v>3.048</v>
       </c>
       <c r="C9" t="n">
-        <v>4.938000000000001</v>
+        <v>4.03</v>
       </c>
       <c r="D9" t="n">
-        <v>5.962000000000001</v>
+        <v>5.322</v>
       </c>
       <c r="E9" t="n">
-        <v>7.222</v>
+        <v>6.228</v>
       </c>
       <c r="F9" t="n">
-        <v>8.997999999999999</v>
+        <v>7.692</v>
       </c>
       <c r="G9" t="n">
-        <v>10.604</v>
+        <v>9.093999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>10.878</v>
+        <v>9.284000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>12.842</v>
+        <v>10.854</v>
       </c>
       <c r="J9" t="n">
-        <v>13.434</v>
+        <v>11.584</v>
       </c>
       <c r="K9" t="n">
-        <v>13.716</v>
+        <v>12.022</v>
       </c>
       <c r="L9" t="n">
-        <v>15.076</v>
+        <v>13.19</v>
       </c>
       <c r="M9" t="n">
-        <v>16.53</v>
+        <v>13.948</v>
       </c>
       <c r="N9" t="n">
-        <v>16.962</v>
+        <v>14.874</v>
       </c>
       <c r="O9" t="n">
-        <v>19.422</v>
+        <v>17.054</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3.394</v>
+        <v>2.714</v>
       </c>
       <c r="B10" t="n">
-        <v>4.557</v>
+        <v>3.654</v>
       </c>
       <c r="C10" t="n">
-        <v>5.502</v>
+        <v>4.938000000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>6.882</v>
+        <v>5.962000000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>8.418000000000001</v>
+        <v>7.222</v>
       </c>
       <c r="F10" t="n">
-        <v>10.274</v>
+        <v>8.997999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>11.948</v>
+        <v>10.604</v>
       </c>
       <c r="H10" t="n">
-        <v>12.464</v>
+        <v>10.878</v>
       </c>
       <c r="I10" t="n">
-        <v>14.664</v>
+        <v>12.842</v>
       </c>
       <c r="J10" t="n">
-        <v>15.402</v>
+        <v>13.434</v>
       </c>
       <c r="K10" t="n">
-        <v>15.706</v>
+        <v>13.716</v>
       </c>
       <c r="L10" t="n">
-        <v>17.502</v>
+        <v>15.076</v>
       </c>
       <c r="M10" t="n">
-        <v>19.034</v>
+        <v>16.53</v>
       </c>
       <c r="N10" t="n">
-        <v>19.602</v>
+        <v>16.962</v>
       </c>
       <c r="O10" t="n">
-        <v>21.962</v>
+        <v>19.422</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>4.2525</v>
+        <v>3.394</v>
       </c>
       <c r="B11" t="n">
-        <v>5.9275</v>
+        <v>4.557</v>
       </c>
       <c r="C11" t="n">
-        <v>6.703999999999999</v>
+        <v>5.502</v>
       </c>
       <c r="D11" t="n">
-        <v>7.872</v>
+        <v>6.882</v>
       </c>
       <c r="E11" t="n">
-        <v>9.706</v>
+        <v>8.418000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>12.092</v>
+        <v>10.274</v>
       </c>
       <c r="G11" t="n">
-        <v>13.944</v>
+        <v>11.948</v>
       </c>
       <c r="H11" t="n">
-        <v>14.568</v>
+        <v>12.464</v>
       </c>
       <c r="I11" t="n">
-        <v>17.114</v>
+        <v>14.664</v>
       </c>
       <c r="J11" t="n">
-        <v>18.2</v>
+        <v>15.402</v>
       </c>
       <c r="K11" t="n">
-        <v>18.05</v>
+        <v>15.706</v>
       </c>
       <c r="L11" t="n">
-        <v>20.14</v>
+        <v>17.502</v>
       </c>
       <c r="M11" t="n">
-        <v>21.934</v>
+        <v>19.034</v>
       </c>
       <c r="N11" t="n">
-        <v>22.542</v>
+        <v>19.602</v>
       </c>
       <c r="O11" t="n">
-        <v>24.644</v>
+        <v>21.962</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>4.77725</v>
+        <v>4.2525</v>
       </c>
       <c r="B12" t="n">
-        <v>7.364749999999999</v>
+        <v>5.9275</v>
       </c>
       <c r="C12" t="n">
-        <v>8.163</v>
+        <v>6.703999999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>8.976000000000003</v>
+        <v>7.872</v>
       </c>
       <c r="E12" t="n">
-        <v>11.246</v>
+        <v>9.706</v>
       </c>
       <c r="F12" t="n">
-        <v>13.765</v>
+        <v>12.092</v>
       </c>
       <c r="G12" t="n">
-        <v>15.922</v>
+        <v>13.944</v>
       </c>
       <c r="H12" t="n">
-        <v>16.654</v>
+        <v>14.568</v>
       </c>
       <c r="I12" t="n">
-        <v>19.402</v>
+        <v>17.114</v>
       </c>
       <c r="J12" t="n">
-        <v>20.59</v>
+        <v>18.2</v>
       </c>
       <c r="K12" t="n">
-        <v>20.554</v>
+        <v>18.05</v>
       </c>
       <c r="L12" t="n">
-        <v>22.982</v>
+        <v>20.14</v>
       </c>
       <c r="M12" t="n">
-        <v>25.287</v>
+        <v>21.934</v>
       </c>
       <c r="N12" t="n">
-        <v>26.025</v>
+        <v>22.542</v>
       </c>
       <c r="O12" t="n">
-        <v>27.85</v>
+        <v>24.644</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5.039624999999999</v>
+        <v>4.77725</v>
       </c>
       <c r="B13" t="n">
-        <v>8.047374999999999</v>
+        <v>7.364749999999999</v>
       </c>
       <c r="C13" t="n">
-        <v>9.493</v>
+        <v>8.163</v>
       </c>
       <c r="D13" t="n">
-        <v>10.441</v>
+        <v>8.976000000000003</v>
       </c>
       <c r="E13" t="n">
-        <v>12.857</v>
+        <v>11.246</v>
       </c>
       <c r="F13" t="n">
-        <v>15.897</v>
+        <v>13.765</v>
       </c>
       <c r="G13" t="n">
-        <v>18.07</v>
+        <v>15.922</v>
       </c>
       <c r="H13" t="n">
-        <v>19.131</v>
+        <v>16.654</v>
       </c>
       <c r="I13" t="n">
-        <v>22.04</v>
+        <v>19.402</v>
       </c>
       <c r="J13" t="n">
-        <v>23.305</v>
+        <v>20.59</v>
       </c>
       <c r="K13" t="n">
-        <v>23.508</v>
+        <v>20.554</v>
       </c>
       <c r="L13" t="n">
-        <v>26.18</v>
+        <v>22.982</v>
       </c>
       <c r="M13" t="n">
-        <v>28.756</v>
+        <v>25.287</v>
       </c>
       <c r="N13" t="n">
-        <v>29.3495</v>
+        <v>26.025</v>
       </c>
       <c r="O13" t="n">
-        <v>31.354</v>
+        <v>27.85</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>5.170812400000001</v>
+        <v>5.039624999999999</v>
       </c>
       <c r="B14" t="n">
-        <v>8.1046874</v>
+        <v>8.047374999999999</v>
       </c>
       <c r="C14" t="n">
-        <v>9.847</v>
+        <v>9.493</v>
       </c>
       <c r="D14" t="n">
-        <v>11.7825</v>
+        <v>10.441</v>
       </c>
       <c r="E14" t="n">
-        <v>14.1885</v>
+        <v>12.857</v>
       </c>
       <c r="F14" t="n">
-        <v>17.2245</v>
+        <v>15.897</v>
       </c>
       <c r="G14" t="n">
-        <v>19.742</v>
+        <v>18.07</v>
       </c>
       <c r="H14" t="n">
-        <v>20.716</v>
+        <v>19.131</v>
       </c>
       <c r="I14" t="n">
-        <v>24.435</v>
+        <v>22.04</v>
       </c>
       <c r="J14" t="n">
-        <v>25.631</v>
+        <v>23.305</v>
       </c>
       <c r="K14" t="n">
-        <v>26.219</v>
+        <v>23.508</v>
       </c>
       <c r="L14" t="n">
-        <v>28.95600000000001</v>
+        <v>26.18</v>
       </c>
       <c r="M14" t="n">
-        <v>31.583</v>
+        <v>28.756</v>
       </c>
       <c r="N14" t="n">
-        <v>32.20399999999999</v>
+        <v>29.3495</v>
       </c>
       <c r="O14" t="n">
-        <v>34.506</v>
+        <v>31.354</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>5.2649062</v>
+        <v>5.170812400000001</v>
       </c>
       <c r="B15" t="n">
-        <v>7.8683436</v>
+        <v>8.1046874</v>
       </c>
       <c r="C15" t="n">
-        <v>9.91</v>
+        <v>9.847</v>
       </c>
       <c r="D15" t="n">
-        <v>12.848</v>
+        <v>11.7825</v>
       </c>
       <c r="E15" t="n">
-        <v>15.608</v>
+        <v>14.1885</v>
       </c>
       <c r="F15" t="n">
-        <v>18.612</v>
+        <v>17.2245</v>
       </c>
       <c r="G15" t="n">
-        <v>21.296</v>
+        <v>19.742</v>
       </c>
       <c r="H15" t="n">
-        <v>22.564</v>
+        <v>20.716</v>
       </c>
       <c r="I15" t="n">
-        <v>25.9785</v>
+        <v>24.435</v>
       </c>
       <c r="J15" t="n">
-        <v>27.484</v>
+        <v>25.631</v>
       </c>
       <c r="K15" t="n">
-        <v>28.546</v>
+        <v>26.219</v>
       </c>
       <c r="L15" t="n">
-        <v>31.194</v>
+        <v>28.95600000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>33.982</v>
+        <v>31.583</v>
       </c>
       <c r="N15" t="n">
-        <v>35.158</v>
+        <v>32.20399999999999</v>
       </c>
       <c r="O15" t="n">
-        <v>37.354</v>
+        <v>34.506</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>5.454</v>
+        <v>5.2649062</v>
       </c>
       <c r="B16" t="n">
-        <v>8.244</v>
+        <v>7.8683436</v>
       </c>
       <c r="C16" t="n">
-        <v>10.484</v>
+        <v>9.91</v>
       </c>
       <c r="D16" t="n">
-        <v>12.988</v>
+        <v>12.848</v>
       </c>
       <c r="E16" t="n">
-        <v>16.198</v>
+        <v>15.608</v>
       </c>
       <c r="F16" t="n">
-        <v>19.01</v>
+        <v>18.612</v>
       </c>
       <c r="G16" t="n">
-        <v>21.65</v>
+        <v>21.296</v>
       </c>
       <c r="H16" t="n">
-        <v>23.326</v>
+        <v>22.564</v>
       </c>
       <c r="I16" t="n">
-        <v>26.678</v>
+        <v>25.9785</v>
       </c>
       <c r="J16" t="n">
-        <v>28.078</v>
+        <v>27.484</v>
       </c>
       <c r="K16" t="n">
-        <v>29.614</v>
+        <v>28.546</v>
       </c>
       <c r="L16" t="n">
-        <v>32.282</v>
+        <v>31.194</v>
       </c>
       <c r="M16" t="n">
-        <v>34.872</v>
+        <v>33.982</v>
       </c>
       <c r="N16" t="n">
-        <v>36.956</v>
+        <v>35.158</v>
       </c>
       <c r="O16" t="n">
-        <v>39.35</v>
+        <v>37.354</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>5.59</v>
+        <v>5.454</v>
       </c>
       <c r="B17" t="n">
-        <v>8.558</v>
+        <v>8.244</v>
       </c>
       <c r="C17" t="n">
-        <v>10.828</v>
+        <v>10.484</v>
       </c>
       <c r="D17" t="n">
-        <v>13.458</v>
+        <v>12.988</v>
       </c>
       <c r="E17" t="n">
-        <v>16.644</v>
+        <v>16.198</v>
       </c>
       <c r="F17" t="n">
-        <v>19.514</v>
+        <v>19.01</v>
       </c>
       <c r="G17" t="n">
-        <v>21.828</v>
+        <v>21.65</v>
       </c>
       <c r="H17" t="n">
-        <v>24.014</v>
+        <v>23.326</v>
       </c>
       <c r="I17" t="n">
-        <v>26.668</v>
+        <v>26.678</v>
       </c>
       <c r="J17" t="n">
-        <v>28.584</v>
+        <v>28.078</v>
       </c>
       <c r="K17" t="n">
-        <v>30.654</v>
+        <v>29.614</v>
       </c>
       <c r="L17" t="n">
-        <v>32.866</v>
+        <v>32.282</v>
       </c>
       <c r="M17" t="n">
-        <v>35.096</v>
+        <v>34.872</v>
       </c>
       <c r="N17" t="n">
-        <v>37.882</v>
+        <v>36.956</v>
       </c>
       <c r="O17" t="n">
-        <v>40.41799999999999</v>
+        <v>39.35</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>5.454</v>
+        <v>5.59</v>
       </c>
       <c r="B18" t="n">
-        <v>8.071999999999999</v>
+        <v>8.558</v>
       </c>
       <c r="C18" t="n">
-        <v>10.614</v>
+        <v>10.828</v>
       </c>
       <c r="D18" t="n">
-        <v>12.84</v>
+        <v>13.458</v>
       </c>
       <c r="E18" t="n">
-        <v>16.126</v>
+        <v>16.644</v>
       </c>
       <c r="F18" t="n">
-        <v>18.712</v>
+        <v>19.514</v>
       </c>
       <c r="G18" t="n">
-        <v>20.734</v>
+        <v>21.828</v>
       </c>
       <c r="H18" t="n">
-        <v>23.072</v>
+        <v>24.014</v>
       </c>
       <c r="I18" t="n">
-        <v>25.674</v>
+        <v>26.668</v>
       </c>
       <c r="J18" t="n">
-        <v>27.488</v>
+        <v>28.584</v>
       </c>
       <c r="K18" t="n">
-        <v>30.018</v>
+        <v>30.654</v>
       </c>
       <c r="L18" t="n">
-        <v>31.784</v>
+        <v>32.866</v>
       </c>
       <c r="M18" t="n">
-        <v>33.812</v>
+        <v>35.096</v>
       </c>
       <c r="N18" t="n">
-        <v>36.924</v>
+        <v>37.882</v>
       </c>
       <c r="O18" t="n">
-        <v>39.976</v>
+        <v>40.41799999999999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>5.13</v>
+        <v>5.454</v>
       </c>
       <c r="B19" t="n">
-        <v>7.798</v>
+        <v>8.071999999999999</v>
       </c>
       <c r="C19" t="n">
-        <v>10.454</v>
+        <v>10.614</v>
       </c>
       <c r="D19" t="n">
-        <v>12.276</v>
+        <v>12.84</v>
       </c>
       <c r="E19" t="n">
-        <v>15.484</v>
+        <v>16.126</v>
       </c>
       <c r="F19" t="n">
-        <v>17.86</v>
+        <v>18.712</v>
       </c>
       <c r="G19" t="n">
-        <v>19.786</v>
+        <v>20.734</v>
       </c>
       <c r="H19" t="n">
-        <v>22.33</v>
+        <v>23.072</v>
       </c>
       <c r="I19" t="n">
-        <v>24.21</v>
+        <v>25.674</v>
       </c>
       <c r="J19" t="n">
-        <v>25.848</v>
+        <v>27.488</v>
       </c>
       <c r="K19" t="n">
-        <v>29.064</v>
+        <v>30.018</v>
       </c>
       <c r="L19" t="n">
-        <v>30.146</v>
+        <v>31.784</v>
       </c>
       <c r="M19" t="n">
-        <v>32.146</v>
+        <v>33.812</v>
       </c>
       <c r="N19" t="n">
-        <v>35.384</v>
+        <v>36.924</v>
       </c>
       <c r="O19" t="n">
-        <v>38.59400000000001</v>
+        <v>39.976</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>4.912000000000001</v>
+        <v>5.13</v>
       </c>
       <c r="B20" t="n">
-        <v>7.278</v>
+        <v>7.798</v>
       </c>
       <c r="C20" t="n">
-        <v>9.867999999999999</v>
+        <v>10.454</v>
       </c>
       <c r="D20" t="n">
-        <v>11.114</v>
+        <v>12.276</v>
       </c>
       <c r="E20" t="n">
-        <v>13.95</v>
+        <v>15.484</v>
       </c>
       <c r="F20" t="n">
-        <v>16.412</v>
+        <v>17.86</v>
       </c>
       <c r="G20" t="n">
-        <v>18.03</v>
+        <v>19.786</v>
       </c>
       <c r="H20" t="n">
-        <v>20.296</v>
+        <v>22.33</v>
       </c>
       <c r="I20" t="n">
-        <v>21.788</v>
+        <v>24.21</v>
       </c>
       <c r="J20" t="n">
-        <v>23.286</v>
+        <v>25.848</v>
       </c>
       <c r="K20" t="n">
-        <v>26.67</v>
+        <v>29.064</v>
       </c>
       <c r="L20" t="n">
-        <v>27.46</v>
+        <v>30.146</v>
       </c>
       <c r="M20" t="n">
-        <v>29.05</v>
+        <v>32.146</v>
       </c>
       <c r="N20" t="n">
-        <v>32.394</v>
+        <v>35.384</v>
       </c>
       <c r="O20" t="n">
-        <v>35.58800000000001</v>
+        <v>38.59400000000001</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>4.532</v>
+        <v>4.912000000000001</v>
       </c>
       <c r="B21" t="n">
-        <v>6.846000000000001</v>
+        <v>7.278</v>
       </c>
       <c r="C21" t="n">
-        <v>8.516</v>
+        <v>9.867999999999999</v>
       </c>
       <c r="D21" t="n">
-        <v>10.138</v>
+        <v>11.114</v>
       </c>
       <c r="E21" t="n">
-        <v>12.68</v>
+        <v>13.95</v>
       </c>
       <c r="F21" t="n">
-        <v>14.636</v>
+        <v>16.412</v>
       </c>
       <c r="G21" t="n">
-        <v>16.174</v>
+        <v>18.03</v>
       </c>
       <c r="H21" t="n">
-        <v>18.126</v>
+        <v>20.296</v>
       </c>
       <c r="I21" t="n">
-        <v>19.26</v>
+        <v>21.788</v>
       </c>
       <c r="J21" t="n">
-        <v>20.548</v>
+        <v>23.286</v>
       </c>
       <c r="K21" t="n">
-        <v>23.598</v>
+        <v>26.67</v>
       </c>
       <c r="L21" t="n">
-        <v>24.18</v>
+        <v>27.46</v>
       </c>
       <c r="M21" t="n">
-        <v>25.428</v>
+        <v>29.05</v>
       </c>
       <c r="N21" t="n">
-        <v>28.724</v>
+        <v>32.394</v>
       </c>
       <c r="O21" t="n">
-        <v>31.744</v>
+        <v>35.58800000000001</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>4.092000000000001</v>
+        <v>4.532</v>
       </c>
       <c r="B22" t="n">
-        <v>6.34</v>
+        <v>6.846000000000001</v>
       </c>
       <c r="C22" t="n">
-        <v>7.808</v>
+        <v>8.516</v>
       </c>
       <c r="D22" t="n">
-        <v>9.16</v>
+        <v>10.138</v>
       </c>
       <c r="E22" t="n">
-        <v>11.212</v>
+        <v>12.68</v>
       </c>
       <c r="F22" t="n">
-        <v>13.224</v>
+        <v>14.636</v>
       </c>
       <c r="G22" t="n">
-        <v>14.422</v>
+        <v>16.174</v>
       </c>
       <c r="H22" t="n">
-        <v>16.102</v>
+        <v>18.126</v>
       </c>
       <c r="I22" t="n">
-        <v>17.114</v>
+        <v>19.26</v>
       </c>
       <c r="J22" t="n">
-        <v>18.444</v>
+        <v>20.548</v>
       </c>
       <c r="K22" t="n">
-        <v>20.96</v>
+        <v>23.598</v>
       </c>
       <c r="L22" t="n">
-        <v>21.236</v>
+        <v>24.18</v>
       </c>
       <c r="M22" t="n">
-        <v>22.45</v>
+        <v>25.428</v>
       </c>
       <c r="N22" t="n">
-        <v>24.862</v>
+        <v>28.724</v>
       </c>
       <c r="O22" t="n">
-        <v>27.992</v>
+        <v>31.744</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3.728</v>
+        <v>4.092000000000001</v>
       </c>
       <c r="B23" t="n">
-        <v>5.712000000000001</v>
+        <v>6.34</v>
       </c>
       <c r="C23" t="n">
-        <v>6.961999999999999</v>
+        <v>7.808</v>
       </c>
       <c r="D23" t="n">
-        <v>8.096</v>
+        <v>9.16</v>
       </c>
       <c r="E23" t="n">
-        <v>9.988</v>
+        <v>11.212</v>
       </c>
       <c r="F23" t="n">
-        <v>11.438</v>
+        <v>13.224</v>
       </c>
       <c r="G23" t="n">
-        <v>12.732</v>
+        <v>14.422</v>
       </c>
       <c r="H23" t="n">
-        <v>14.094</v>
+        <v>16.102</v>
       </c>
       <c r="I23" t="n">
-        <v>15.044</v>
+        <v>17.114</v>
       </c>
       <c r="J23" t="n">
-        <v>15.978</v>
+        <v>18.444</v>
       </c>
       <c r="K23" t="n">
-        <v>18.158</v>
+        <v>20.96</v>
       </c>
       <c r="L23" t="n">
-        <v>18.582</v>
+        <v>21.236</v>
       </c>
       <c r="M23" t="n">
-        <v>19.538</v>
+        <v>22.45</v>
       </c>
       <c r="N23" t="n">
-        <v>21.754</v>
+        <v>24.862</v>
       </c>
       <c r="O23" t="n">
-        <v>24.478</v>
+        <v>27.992</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3.398000000000001</v>
+        <v>3.728</v>
       </c>
       <c r="B24" t="n">
-        <v>4.782</v>
+        <v>5.712000000000001</v>
       </c>
       <c r="C24" t="n">
-        <v>6.15</v>
+        <v>6.961999999999999</v>
       </c>
       <c r="D24" t="n">
-        <v>7.081999999999999</v>
+        <v>8.096</v>
       </c>
       <c r="E24" t="n">
-        <v>8.726000000000001</v>
+        <v>9.988</v>
       </c>
       <c r="F24" t="n">
-        <v>10.002</v>
+        <v>11.438</v>
       </c>
       <c r="G24" t="n">
-        <v>11.26</v>
+        <v>12.732</v>
       </c>
       <c r="H24" t="n">
-        <v>12.338</v>
+        <v>14.094</v>
       </c>
       <c r="I24" t="n">
-        <v>13.096</v>
+        <v>15.044</v>
       </c>
       <c r="J24" t="n">
-        <v>13.832</v>
+        <v>15.978</v>
       </c>
       <c r="K24" t="n">
-        <v>15.706</v>
+        <v>18.158</v>
       </c>
       <c r="L24" t="n">
-        <v>16.324</v>
+        <v>18.582</v>
       </c>
       <c r="M24" t="n">
-        <v>16.89</v>
+        <v>19.538</v>
       </c>
       <c r="N24" t="n">
-        <v>19.022</v>
+        <v>21.754</v>
       </c>
       <c r="O24" t="n">
-        <v>21.192</v>
+        <v>24.478</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3.092</v>
+        <v>3.398000000000001</v>
       </c>
       <c r="B25" t="n">
-        <v>4.406</v>
+        <v>4.782</v>
       </c>
       <c r="C25" t="n">
-        <v>5.182</v>
+        <v>6.15</v>
       </c>
       <c r="D25" t="n">
-        <v>6.258</v>
+        <v>7.081999999999999</v>
       </c>
       <c r="E25" t="n">
-        <v>7.712000000000001</v>
+        <v>8.726000000000001</v>
       </c>
       <c r="F25" t="n">
-        <v>8.747999999999999</v>
+        <v>10.002</v>
       </c>
       <c r="G25" t="n">
-        <v>9.832000000000001</v>
+        <v>11.26</v>
       </c>
       <c r="H25" t="n">
-        <v>10.918</v>
+        <v>12.338</v>
       </c>
       <c r="I25" t="n">
-        <v>11.634</v>
+        <v>13.096</v>
       </c>
       <c r="J25" t="n">
-        <v>12.184</v>
+        <v>13.832</v>
       </c>
       <c r="K25" t="n">
-        <v>13.756</v>
+        <v>15.706</v>
       </c>
       <c r="L25" t="n">
-        <v>13.972</v>
+        <v>16.324</v>
       </c>
       <c r="M25" t="n">
-        <v>14.556</v>
+        <v>16.89</v>
       </c>
       <c r="N25" t="n">
-        <v>16.324</v>
+        <v>19.022</v>
       </c>
       <c r="O25" t="n">
-        <v>18.146</v>
+        <v>21.192</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3</v>
+        <v>3.092</v>
       </c>
       <c r="B26" t="n">
-        <v>4.014</v>
+        <v>4.406</v>
       </c>
       <c r="C26" t="n">
-        <v>4.715999999999999</v>
+        <v>5.182</v>
       </c>
       <c r="D26" t="n">
-        <v>5.465999999999999</v>
+        <v>6.258</v>
       </c>
       <c r="E26" t="n">
-        <v>6.906000000000001</v>
+        <v>7.712000000000001</v>
       </c>
       <c r="F26" t="n">
-        <v>7.863999999999999</v>
+        <v>8.747999999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>8.704000000000001</v>
+        <v>9.832000000000001</v>
       </c>
       <c r="H26" t="n">
-        <v>9.58</v>
+        <v>10.918</v>
       </c>
       <c r="I26" t="n">
-        <v>10.326</v>
+        <v>11.634</v>
       </c>
       <c r="J26" t="n">
-        <v>10.588</v>
+        <v>12.184</v>
       </c>
       <c r="K26" t="n">
-        <v>11.812</v>
+        <v>13.756</v>
       </c>
       <c r="L26" t="n">
-        <v>11.99</v>
+        <v>13.972</v>
       </c>
       <c r="M26" t="n">
-        <v>12.41</v>
+        <v>14.556</v>
       </c>
       <c r="N26" t="n">
-        <v>13.63</v>
+        <v>16.324</v>
       </c>
       <c r="O26" t="n">
-        <v>15.236</v>
+        <v>18.146</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2.616</v>
+        <v>3</v>
       </c>
       <c r="B27" t="n">
-        <v>3.278</v>
+        <v>4.014</v>
       </c>
       <c r="C27" t="n">
-        <v>4.236</v>
+        <v>4.715999999999999</v>
       </c>
       <c r="D27" t="n">
-        <v>4.659999999999999</v>
+        <v>5.465999999999999</v>
       </c>
       <c r="E27" t="n">
-        <v>5.822000000000001</v>
+        <v>6.906000000000001</v>
       </c>
       <c r="F27" t="n">
-        <v>6.736</v>
+        <v>7.863999999999999</v>
       </c>
       <c r="G27" t="n">
-        <v>7.595999999999999</v>
+        <v>8.704000000000001</v>
       </c>
       <c r="H27" t="n">
-        <v>8.097999999999999</v>
+        <v>9.58</v>
       </c>
       <c r="I27" t="n">
-        <v>8.702000000000002</v>
+        <v>10.326</v>
       </c>
       <c r="J27" t="n">
-        <v>9.018000000000001</v>
+        <v>10.588</v>
       </c>
       <c r="K27" t="n">
-        <v>10.098</v>
+        <v>11.812</v>
       </c>
       <c r="L27" t="n">
-        <v>10.396</v>
+        <v>11.99</v>
       </c>
       <c r="M27" t="n">
-        <v>10.856</v>
+        <v>12.41</v>
       </c>
       <c r="N27" t="n">
-        <v>11.846</v>
+        <v>13.63</v>
       </c>
       <c r="O27" t="n">
-        <v>13.336</v>
+        <v>15.236</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2.368</v>
+        <v>2.616</v>
       </c>
       <c r="B28" t="n">
-        <v>2.992</v>
+        <v>3.278</v>
       </c>
       <c r="C28" t="n">
-        <v>3.808</v>
+        <v>4.236</v>
       </c>
       <c r="D28" t="n">
-        <v>4.198</v>
+        <v>4.659999999999999</v>
       </c>
       <c r="E28" t="n">
-        <v>5.13</v>
+        <v>5.822000000000001</v>
       </c>
       <c r="F28" t="n">
-        <v>5.714</v>
+        <v>6.736</v>
       </c>
       <c r="G28" t="n">
-        <v>6.572000000000001</v>
+        <v>7.595999999999999</v>
       </c>
       <c r="H28" t="n">
-        <v>6.934</v>
+        <v>8.097999999999999</v>
       </c>
       <c r="I28" t="n">
-        <v>7.654000000000001</v>
+        <v>8.702000000000002</v>
       </c>
       <c r="J28" t="n">
-        <v>7.736000000000002</v>
+        <v>9.018000000000001</v>
       </c>
       <c r="K28" t="n">
-        <v>8.81</v>
+        <v>10.098</v>
       </c>
       <c r="L28" t="n">
-        <v>9.203999999999999</v>
+        <v>10.396</v>
       </c>
       <c r="M28" t="n">
-        <v>9.423999999999999</v>
+        <v>10.856</v>
       </c>
       <c r="N28" t="n">
-        <v>10.33</v>
+        <v>11.846</v>
       </c>
       <c r="O28" t="n">
-        <v>11.07</v>
+        <v>13.336</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
+        <v>2.368</v>
+      </c>
+      <c r="B29" t="n">
+        <v>2.992</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3.808</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4.198</v>
+      </c>
+      <c r="E29" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5.714</v>
+      </c>
+      <c r="G29" t="n">
+        <v>6.572000000000001</v>
+      </c>
+      <c r="H29" t="n">
+        <v>6.934</v>
+      </c>
+      <c r="I29" t="n">
+        <v>7.654000000000001</v>
+      </c>
+      <c r="J29" t="n">
+        <v>7.736000000000002</v>
+      </c>
+      <c r="K29" t="n">
+        <v>8.81</v>
+      </c>
+      <c r="L29" t="n">
+        <v>9.203999999999999</v>
+      </c>
+      <c r="M29" t="n">
+        <v>9.423999999999999</v>
+      </c>
+      <c r="N29" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="O29" t="n">
+        <v>11.07</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
         <v>1.93</v>
       </c>
-      <c r="B29" t="n">
+      <c r="B30" t="n">
         <v>2.706</v>
       </c>
-      <c r="C29" t="n">
+      <c r="C30" t="n">
         <v>3.18</v>
       </c>
-      <c r="D29" t="n">
+      <c r="D30" t="n">
         <v>3.582</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E30" t="n">
         <v>4.198</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F30" t="n">
         <v>4.668</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G30" t="n">
         <v>5.497999999999999</v>
       </c>
-      <c r="H29" t="n">
+      <c r="H30" t="n">
         <v>5.642</v>
       </c>
-      <c r="I29" t="n">
+      <c r="I30" t="n">
         <v>6.178</v>
       </c>
-      <c r="J29" t="n">
+      <c r="J30" t="n">
         <v>6.286</v>
       </c>
-      <c r="K29" t="n">
+      <c r="K30" t="n">
         <v>7.025999999999999</v>
       </c>
-      <c r="L29" t="n">
+      <c r="L30" t="n">
         <v>7.544</v>
       </c>
-      <c r="M29" t="n">
+      <c r="M30" t="n">
         <v>7.718000000000001</v>
       </c>
-      <c r="N29" t="n">
+      <c r="N30" t="n">
         <v>8.24</v>
       </c>
-      <c r="O29" t="n">
+      <c r="O30" t="n">
         <v>8.914</v>
       </c>
     </row>

</xml_diff>